<commit_message>
feat: prevent stale calculations from producing pass verdicts
</commit_message>
<xml_diff>
--- a/tests/fixtures/clean.xlsx
+++ b/tests/fixtures/clean.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Inputs" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="Provisions" sheetId="2" state="visible" r:id="rId4"/>
   </sheets>
-  <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
+  <calcPr calcId="191029" calcMode="auto" fullCalcOnLoad="1"/>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="ExcelA1"/>
@@ -92,12 +92,16 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -297,12 +301,12 @@
   <sheetFormatPr defaultColWidth="8.5078125" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="n">
+      <c r="A1" s="1" t="n">
         <v>100</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="n">
+      <c r="A2" s="1" t="n">
         <v>200</v>
       </c>
     </row>
@@ -326,35 +330,35 @@
   <sheetFormatPr defaultColWidth="8.5078125" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C1" s="0" t="n">
+      <c r="C1" s="1" t="n">
         <v>10</v>
       </c>
-      <c r="D1" s="0" t="n">
+      <c r="D1" s="1" t="n">
         <f aca="false">Inputs!A1*2</f>
         <v>200</v>
       </c>
-      <c r="E1" s="0" t="n">
+      <c r="E1" s="1" t="n">
         <f aca="false">C5+D1</f>
         <v>300</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C2" s="0" t="n">
+      <c r="C2" s="1" t="n">
         <v>20</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C3" s="0" t="n">
+      <c r="C3" s="1" t="n">
         <v>30</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C4" s="0" t="n">
+      <c r="C4" s="1" t="n">
         <v>40</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C5" s="1" t="n">
+      <c r="C5" s="2" t="n">
         <f aca="false">SUM(C1:C4)</f>
         <v>100</v>
       </c>

</xml_diff>